<commit_message>
Actualizar líderes y códigos de contratos
</commit_message>
<xml_diff>
--- a/database/Directorio_Colbeef.xlsx
+++ b/database/Directorio_Colbeef.xlsx
@@ -1236,12 +1236,12 @@
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
         <is>
-          <t>ASUNTOS CORPORATIVOS</t>
+          <t>DIRECCION DE ASUNTOS CORPORATIVOS</t>
         </is>
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>DIRECCION ASUNTOS CORPORATIVOS</t>
+          <t>JURIDICA</t>
         </is>
       </c>
       <c r="C35" s="3" t="inlineStr">

</xml_diff>